<commit_message>
feat(pro-v6): Upgrade PRO bot to V6 Dual-Engine (Hybrid 65F Trend & 77F Reversal), active execution, responsive mobile layout, and dynamic statistics sync
</commit_message>
<xml_diff>
--- a/Evaluasi_Skenario_Trade.xlsx
+++ b/Evaluasi_Skenario_Trade.xlsx
@@ -649,10 +649,10 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C5" s="5" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>9</v>
@@ -661,25 +661,25 @@
         <v>1</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>73.7</v>
+        <v>73.2</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>34.99</v>
+        <v>32.84</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>0.92</v>
+        <v>0.8</v>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>[28/10 Win]</t>
+          <t>[30/10 Win]</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>[9/10 Loss]</t>
+          <t>[10/10 Loss]</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
@@ -709,7 +709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB42"/>
+  <dimension ref="A1:AB45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -5459,6 +5459,366 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" s="4" t="n">
+        <v>2670573269</v>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09 21:00:01</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09 21:22:13</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>4190.552</v>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>4184.4</v>
+      </c>
+      <c r="I43" s="4" t="n">
+        <v>-61.5</v>
+      </c>
+      <c r="J43" s="4" t="n">
+        <v>-6.15</v>
+      </c>
+      <c r="K43" s="9" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM v5.2 SMC/DXY M15 (65 Fitur)</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>GENERAL_ENTRY</t>
+        </is>
+      </c>
+      <c r="N43" s="4" t="inlineStr">
+        <is>
+          <t>ZONA_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="O43" s="4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P43" s="4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="Q43" s="4" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="R43" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="S43" s="4" t="inlineStr">
+        <is>
+          <t>❌ [LOSS — Analisis Kesalahan]: Stop Loss $4184.40 tersentuh — harga bergerak 61.5 pip melawan posisi dalam 22m 12d | Keyakinan model di batas bawah (50.0%) — entry berisiko tanpa konfluensi penuh.</t>
+        </is>
+      </c>
+      <c r="T43" s="4" t="inlineStr">
+        <is>
+          <t>Untuk skenario GENERAL_ENTRY: Pastikan konfluensi H4 searah sebelum entry. SL minimal 35-50 pip dari entry. Hindari entry jika probabilitas model &lt; 62%.</t>
+        </is>
+      </c>
+      <c r="U43" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09 21:22:14</t>
+        </is>
+      </c>
+      <c r="V43" s="4" t="n">
+        <v>4184.28</v>
+      </c>
+      <c r="W43" s="4" t="inlineStr">
+        <is>
+          <t>GAGAL (TIDAK SELARAS)</t>
+        </is>
+      </c>
+      <c r="X43" s="4" t="n">
+        <v>-62.7</v>
+      </c>
+      <c r="Y43" s="4" t="inlineStr">
+        <is>
+          <t>22m 12d</t>
+        </is>
+      </c>
+      <c r="Z43" s="4" t="n">
+        <v>4184.4</v>
+      </c>
+      <c r="AA43" s="4" t="n">
+        <v>4199.4</v>
+      </c>
+      <c r="AB43" s="4" t="inlineStr">
+        <is>
+          <t>Hit Stop Loss (SL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="n">
+        <v>2670966805</v>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09 22:15:00</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09 22:45:48</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>4185.293</v>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>4187.29</v>
+      </c>
+      <c r="I44" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J44" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K44" s="7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM v5.2 SMC/DXY M15 (65 Fitur)</t>
+        </is>
+      </c>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t>GENERAL_ENTRY</t>
+        </is>
+      </c>
+      <c r="N44" s="4" t="inlineStr">
+        <is>
+          <t>ZONA_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="O44" s="4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P44" s="4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="Q44" s="4" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="R44" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="S44" s="4" t="inlineStr">
+        <is>
+          <t>✅ [WIN — Kemenangan Target]: Trailing profit lock berhasil mengamankan +20.0 pip (exit di $4187.29) sebelum harga berbalik | Validasi Model 75M: SELARAS BERHASIL (Close bar-5: $4187.54, deviasi +22.5 pip searah BUY).</t>
+        </is>
+      </c>
+      <c r="T44" s="4" t="inlineStr">
+        <is>
+          <t>Skenario GENERAL_ENTRY terbukti valid (H4=UNKNOWN, DXY=UNKNOWN). Pertahankan konfluensi multi-timeframe dan disiplin hold hingga TP.</t>
+        </is>
+      </c>
+      <c r="U44" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09 22:45:49</t>
+        </is>
+      </c>
+      <c r="V44" s="4" t="n">
+        <v>4187.54</v>
+      </c>
+      <c r="W44" s="4" t="inlineStr">
+        <is>
+          <t>BERHASIL (SELARAS)</t>
+        </is>
+      </c>
+      <c r="X44" s="4" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="Y44" s="4" t="inlineStr">
+        <is>
+          <t>30m 48d</t>
+        </is>
+      </c>
+      <c r="Z44" s="4" t="n">
+        <v>4178.79</v>
+      </c>
+      <c r="AA44" s="4" t="n">
+        <v>4193.79</v>
+      </c>
+      <c r="AB44" s="4" t="inlineStr">
+        <is>
+          <t>Trailing Lock (BEP +$0.20)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="n">
+        <v>2671148498</v>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09 23:00:00</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09 23:19:29</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>XAUUSD</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="F45" s="4" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>4188.831</v>
+      </c>
+      <c r="H45" s="4" t="n">
+        <v>4190.83</v>
+      </c>
+      <c r="I45" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="J45" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K45" s="7" t="inlineStr">
+        <is>
+          <t>WIN</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>LightGBM v5.2 SMC/DXY M15 (65 Fitur)</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>GENERAL_ENTRY</t>
+        </is>
+      </c>
+      <c r="N45" s="4" t="inlineStr">
+        <is>
+          <t>ZONA_UNKNOWN</t>
+        </is>
+      </c>
+      <c r="O45" s="4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="P45" s="4" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="Q45" s="4" t="inlineStr">
+        <is>
+          <t>NORMAL</t>
+        </is>
+      </c>
+      <c r="R45" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="S45" s="4" t="inlineStr">
+        <is>
+          <t>✅ [WIN — Kemenangan Target]: Trailing profit lock berhasil mengamankan +20.0 pip (exit di $4190.83) sebelum harga berbalik | Validasi Model 75M: SELARAS BERHASIL (Close bar-5: $4191.00, deviasi +21.7 pip searah BUY).</t>
+        </is>
+      </c>
+      <c r="T45" s="4" t="inlineStr">
+        <is>
+          <t>Skenario GENERAL_ENTRY terbukti valid (H4=UNKNOWN, DXY=UNKNOWN). Pertahankan konfluensi multi-timeframe dan disiplin hold hingga TP.</t>
+        </is>
+      </c>
+      <c r="U45" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-09 23:19:30</t>
+        </is>
+      </c>
+      <c r="V45" s="4" t="n">
+        <v>4191</v>
+      </c>
+      <c r="W45" s="4" t="inlineStr">
+        <is>
+          <t>BERHASIL (SELARAS)</t>
+        </is>
+      </c>
+      <c r="X45" s="4" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="Y45" s="4" t="inlineStr">
+        <is>
+          <t>19m 29d</t>
+        </is>
+      </c>
+      <c r="Z45" s="4" t="n">
+        <v>4182.33</v>
+      </c>
+      <c r="AA45" s="4" t="n">
+        <v>4197.33</v>
+      </c>
+      <c r="AB45" s="4" t="inlineStr">
+        <is>
+          <t>Trailing Lock (BEP +$0.20)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>